<commit_message>
Corrige erro de validação
</commit_message>
<xml_diff>
--- a/data/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/data/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E118F84-96F8-4B42-BC1D-AA653C707CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{433A4C8B-94C2-4715-8305-9567B0F83086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="1200" windowWidth="15375" windowHeight="7875" xr2:uid="{0026A821-EB11-4024-9CF3-3B7B6690DDA3}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{0026A821-EB11-4024-9CF3-3B7B6690DDA3}"/>
   </bookViews>
   <sheets>
     <sheet name="cabeçalho" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza dados do órgão
</commit_message>
<xml_diff>
--- a/data/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/data/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0F7789-1847-403B-A213-D644DE712791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BCB2070-EE93-4807-BD31-123312156540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="765" yWindow="1350" windowWidth="15375" windowHeight="7875" xr2:uid="{0026A821-EB11-4024-9CF3-3B7B6690DDA3}"/>
+    <workbookView xWindow="1110" yWindow="1695" windowWidth="15375" windowHeight="7875" xr2:uid="{0026A821-EB11-4024-9CF3-3B7B6690DDA3}"/>
   </bookViews>
   <sheets>
     <sheet name="cabeçalho" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>valor_total_projeto</t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>CGE</t>
+  </si>
+  <si>
+    <t>aaaaa</t>
   </si>
 </sst>
 </file>
@@ -447,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69FD87E0-5473-4C09-9099-10625F3EFC64}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -538,6 +541,26 @@
         <v>500000</v>
       </c>
     </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>9288139</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1">
+        <v>500000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>